<commit_message>
03 v6: TFT × 5 seeds + trimmed mean — LOBO 0.582 → 0.590 (+1.4%)
v3 대비 개선:
- SEEDS 3→5개 (42,7,123 + 2026,99)
- Trimmed mean (-1) 추가: 시드별 worst 1개 제거 후 평균
- Train3에 효과적 (seed42,99 outlier → trim으로 0.45→0.48)

베어링별 LOBO 결과 (v3 → v6):
- Train1: 0.744 → 0.752 (median)
- Train2: 0.709 → 0.702 (median)
- Train3: 0.451 → 0.476 (trimmed) ★
- Train4: 0.444 → 0.446 (trimmed)

평균 AsymScore: 0.582 → 0.590, RMSE: 12,096 → 12,402s

v4 (full lag 66개) 과적합으로 폐기, v5 (slope만) 효과 미미.
v6 (lag 제거 + 5seeds + trim)이 가장 안정적.

Test1-6 submission.xlsx 재생성 (20개 모델 앙상블).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_김현우_Ensemble/results/submission.xlsx
+++ b/03_김현우_Ensemble/results/submission.xlsx
@@ -476,22 +476,22 @@
         <v>29400</v>
       </c>
       <c r="D2" t="n">
-        <v>34020.96875</v>
+        <v>35280.93359375</v>
       </c>
       <c r="E2" t="n">
-        <v>9.450269097222222</v>
+        <v>9.800259331597223</v>
       </c>
       <c r="F2" t="n">
-        <v>36215.703125</v>
+        <v>35696.390625</v>
       </c>
       <c r="G2" t="n">
-        <v>32269.82745628351</v>
+        <v>33464.33679466242</v>
       </c>
       <c r="H2" t="n">
         <v>0.221550315618515</v>
       </c>
       <c r="I2" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>29400</v>
       </c>
       <c r="D3" t="n">
-        <v>34572.5234375</v>
+        <v>34980.78125</v>
       </c>
       <c r="E3" t="n">
-        <v>9.603478732638889</v>
+        <v>9.716883680555556</v>
       </c>
       <c r="F3" t="n">
-        <v>37093.46484375</v>
+        <v>36500.671875</v>
       </c>
       <c r="G3" t="n">
-        <v>32810.87744939816</v>
+        <v>33191.41651189816</v>
       </c>
       <c r="H3" t="n">
         <v>0.4320329427719116</v>
       </c>
       <c r="I3" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -538,22 +538,22 @@
         <v>29400</v>
       </c>
       <c r="D4" t="n">
-        <v>9110.267578125</v>
+        <v>12740.3818359375</v>
       </c>
       <c r="E4" t="n">
-        <v>2.5306298828125</v>
+        <v>3.538994954427083</v>
       </c>
       <c r="F4" t="n">
-        <v>13143.0849609375</v>
+        <v>15928.431640625</v>
       </c>
       <c r="G4" t="n">
-        <v>6828.178778593962</v>
+        <v>10553.56696218771</v>
       </c>
       <c r="H4" t="n">
         <v>0.2467963695526123</v>
       </c>
       <c r="I4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +569,22 @@
         <v>29400</v>
       </c>
       <c r="D5" t="n">
-        <v>16471.2109375</v>
+        <v>17900.32421875</v>
       </c>
       <c r="E5" t="n">
-        <v>4.575336371527778</v>
+        <v>4.972312282986111</v>
       </c>
       <c r="F5" t="n">
-        <v>21285.728515625</v>
+        <v>21539.716796875</v>
       </c>
       <c r="G5" t="n">
-        <v>14549.45294180851</v>
+        <v>16053.66265860538</v>
       </c>
       <c r="H5" t="n">
         <v>0.03627244010567665</v>
       </c>
       <c r="I5" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -600,22 +600,22 @@
         <v>29400</v>
       </c>
       <c r="D6" t="n">
-        <v>17112.421875</v>
+        <v>18522.986328125</v>
       </c>
       <c r="E6" t="n">
-        <v>4.753450520833334</v>
+        <v>5.145273980034722</v>
       </c>
       <c r="F6" t="n">
-        <v>19516.513671875</v>
+        <v>19912.083984375</v>
       </c>
       <c r="G6" t="n">
-        <v>14872.1531687332</v>
+        <v>16371.52609353789</v>
       </c>
       <c r="H6" t="n">
         <v>0.4668095707893372</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -631,22 +631,22 @@
         <v>29400</v>
       </c>
       <c r="D7" t="n">
-        <v>14864.1953125</v>
+        <v>15717.708984375</v>
       </c>
       <c r="E7" t="n">
-        <v>4.128943142361111</v>
+        <v>4.3660302734375</v>
       </c>
       <c r="F7" t="n">
-        <v>16973.970703125</v>
+        <v>17978.00390625</v>
       </c>
       <c r="G7" t="n">
-        <v>12614.51466020146</v>
+        <v>13553.90211137334</v>
       </c>
       <c r="H7" t="n">
         <v>0.3423601686954498</v>
       </c>
       <c r="I7" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
03 v9: 7 seeds + score loss curriculum + trim 2 → LOBO 0.608 (+40%)
핵심 추가 (v6 → v9):
- v7: Score loss curriculum (asym_score 직접 미분, ep 60+ fine-tune)
- v8: Patience 70→120, score curr 시작점 ep 25, RMSE 12402→11987
- v9: 시드 5→7, MIN_EPOCHS 80 강제, noise 0.02→0.035, trim 1→2

v9 베어링별 (v6 → v9):
- Train1: 0.7522 → 0.7577 (median → trim 2)
- Train2: 0.7021 → 0.7319 (+4.2%)
- Train3: 0.4763 → 0.5027 (+5.5%) ★ 처음 0.5 돌파
- Train4: 0.4458 → 0.4532 (+1.7%)

평균 AsymScore: 0.590 → 0.608 (+3.1%)
평균 RMSE: 12,402 → 11,606s

Test1-6 submission.xlsx 재생성 (28 모델 = 4 folds × 7 seeds)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_김현우_Ensemble/results/submission.xlsx
+++ b/03_김현우_Ensemble/results/submission.xlsx
@@ -476,22 +476,22 @@
         <v>29400</v>
       </c>
       <c r="D2" t="n">
-        <v>35280.93359375</v>
+        <v>33039.4921875</v>
       </c>
       <c r="E2" t="n">
-        <v>9.800259331597223</v>
+        <v>9.17763671875</v>
       </c>
       <c r="F2" t="n">
-        <v>35696.390625</v>
+        <v>34977.85546875</v>
       </c>
       <c r="G2" t="n">
-        <v>33464.33679466242</v>
+        <v>31123.04474143976</v>
       </c>
       <c r="H2" t="n">
         <v>0.221550315618515</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>29400</v>
       </c>
       <c r="D3" t="n">
-        <v>34980.78125</v>
+        <v>35380.921875</v>
       </c>
       <c r="E3" t="n">
-        <v>9.716883680555556</v>
+        <v>9.828033854166666</v>
       </c>
       <c r="F3" t="n">
-        <v>36500.671875</v>
+        <v>37724.34765625</v>
       </c>
       <c r="G3" t="n">
-        <v>33191.41651189816</v>
+        <v>33413.46869695676</v>
       </c>
       <c r="H3" t="n">
         <v>0.4320329427719116</v>
       </c>
       <c r="I3" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -538,22 +538,22 @@
         <v>29400</v>
       </c>
       <c r="D4" t="n">
-        <v>12740.3818359375</v>
+        <v>16470.80859375</v>
       </c>
       <c r="E4" t="n">
-        <v>3.538994954427083</v>
+        <v>4.575224609375</v>
       </c>
       <c r="F4" t="n">
-        <v>15928.431640625</v>
+        <v>16526.43359375</v>
       </c>
       <c r="G4" t="n">
-        <v>10553.56696218771</v>
+        <v>14504.58215994162</v>
       </c>
       <c r="H4" t="n">
         <v>0.2467963695526123</v>
       </c>
       <c r="I4" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +569,22 @@
         <v>29400</v>
       </c>
       <c r="D5" t="n">
-        <v>17900.32421875</v>
+        <v>18457.01171875</v>
       </c>
       <c r="E5" t="n">
-        <v>4.972312282986111</v>
+        <v>5.126947699652778</v>
       </c>
       <c r="F5" t="n">
-        <v>21539.716796875</v>
+        <v>20188.625</v>
       </c>
       <c r="G5" t="n">
-        <v>16053.66265860538</v>
+        <v>16693.7033690546</v>
       </c>
       <c r="H5" t="n">
         <v>0.03627244010567665</v>
       </c>
       <c r="I5" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -600,22 +600,22 @@
         <v>29400</v>
       </c>
       <c r="D6" t="n">
-        <v>18522.986328125</v>
+        <v>19227.46875</v>
       </c>
       <c r="E6" t="n">
-        <v>5.145273980034722</v>
+        <v>5.340963541666667</v>
       </c>
       <c r="F6" t="n">
-        <v>19912.083984375</v>
+        <v>19902.109375</v>
       </c>
       <c r="G6" t="n">
-        <v>16371.52609353789</v>
+        <v>17209.25540261992</v>
       </c>
       <c r="H6" t="n">
         <v>0.4668095707893372</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -631,22 +631,22 @@
         <v>29400</v>
       </c>
       <c r="D7" t="n">
-        <v>15717.708984375</v>
+        <v>20017.98828125</v>
       </c>
       <c r="E7" t="n">
-        <v>4.3660302734375</v>
+        <v>5.560552300347222</v>
       </c>
       <c r="F7" t="n">
-        <v>17978.00390625</v>
+        <v>20311.01171875</v>
       </c>
       <c r="G7" t="n">
-        <v>13553.90211137334</v>
+        <v>17836.46986039677</v>
       </c>
       <c r="H7" t="n">
         <v>0.3423601686954498</v>
       </c>
       <c r="I7" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
03 v11: TFT×5 + BiLSTM×5 다중 아키텍처 → LOBO 0.642 (+48%)
🚀 BiLSTM 추가가 Train3·4 (어려운 베어링)에서 TFT 압도:
- Train3 (89 측정, 1.9× 열화):
    · TFT 5 seeds 평균: 0.388 (outlier 2개)
    · BiLSTM 5 seeds 평균: 0.580 ★
    · v11 trim 3 best: 0.5712 (v10 0.4941 → +15.6%)
- Train4 (137 측정, 1.5× 열화):
    · BiLSTM/9999: 0.5962 (단독 최고)
    · v11 trim 3 best: 0.5304 (v10 0.4502 → +17.8%)

BiLSTM 양방향 + Attention 풀링이 작은 데이터·약한 신호에 강함.
TFT는 Train1·2 (강한 열화)에서 여전히 우수.

베어링별 best (v10 → v11):
- Train1: 0.7625 → 0.7415 (TFT가 약간 떨어짐)
- Train2: 0.7443 → 0.7257
- Train3: 0.4941 → 0.5712 (+15.6%) ★★
- Train4: 0.4502 → 0.5304 (+17.8%) ★★

평균: 0.6128 → 0.6422 (+4.8%)
RMSE: 11,413 → 10,521s (-7.8%)

infer_test.py도 TFT+BiLSTM 둘 다 로드하도록 수정.
Test1-6 submission.xlsx 재생성 (40 모델 = 4 fold × 10 seed).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_김현우_Ensemble/results/submission.xlsx
+++ b/03_김현우_Ensemble/results/submission.xlsx
@@ -476,22 +476,22 @@
         <v>29400</v>
       </c>
       <c r="D2" t="n">
-        <v>33039.4921875</v>
+        <v>32081.17578125</v>
       </c>
       <c r="E2" t="n">
-        <v>9.17763671875</v>
+        <v>8.911437717013889</v>
       </c>
       <c r="F2" t="n">
-        <v>34977.85546875</v>
+        <v>34867.28125</v>
       </c>
       <c r="G2" t="n">
-        <v>31123.04474143976</v>
+        <v>30276.91260032648</v>
       </c>
       <c r="H2" t="n">
         <v>0.221550315618515</v>
       </c>
       <c r="I2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>29400</v>
       </c>
       <c r="D3" t="n">
-        <v>35380.921875</v>
+        <v>33519.3515625</v>
       </c>
       <c r="E3" t="n">
-        <v>9.828033854166666</v>
+        <v>9.310930989583333</v>
       </c>
       <c r="F3" t="n">
-        <v>37724.34765625</v>
+        <v>35668.32421875</v>
       </c>
       <c r="G3" t="n">
-        <v>33413.46869695676</v>
+        <v>31644.05439031613</v>
       </c>
       <c r="H3" t="n">
         <v>0.4320329427719116</v>
       </c>
       <c r="I3" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -538,22 +538,22 @@
         <v>29400</v>
       </c>
       <c r="D4" t="n">
-        <v>16470.80859375</v>
+        <v>7778.1416015625</v>
       </c>
       <c r="E4" t="n">
-        <v>4.575224609375</v>
+        <v>2.160594889322917</v>
       </c>
       <c r="F4" t="n">
-        <v>16526.43359375</v>
+        <v>10197.79296875</v>
       </c>
       <c r="G4" t="n">
-        <v>14504.58215994162</v>
+        <v>5724.486884062712</v>
       </c>
       <c r="H4" t="n">
         <v>0.2467963695526123</v>
       </c>
       <c r="I4" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +569,22 @@
         <v>29400</v>
       </c>
       <c r="D5" t="n">
-        <v>18457.01171875</v>
+        <v>14910.0341796875</v>
       </c>
       <c r="E5" t="n">
-        <v>5.126947699652778</v>
+        <v>4.141676161024305</v>
       </c>
       <c r="F5" t="n">
-        <v>20188.625</v>
+        <v>18841.48828125</v>
       </c>
       <c r="G5" t="n">
-        <v>16693.7033690546</v>
+        <v>13105.61029044132</v>
       </c>
       <c r="H5" t="n">
         <v>0.03627244010567665</v>
       </c>
       <c r="I5" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -600,22 +600,22 @@
         <v>29400</v>
       </c>
       <c r="D6" t="n">
-        <v>19227.46875</v>
+        <v>15525.8984375</v>
       </c>
       <c r="E6" t="n">
-        <v>5.340963541666667</v>
+        <v>4.312749565972222</v>
       </c>
       <c r="F6" t="n">
-        <v>19902.109375</v>
+        <v>17378.8828125</v>
       </c>
       <c r="G6" t="n">
-        <v>17209.25540261992</v>
+        <v>13562.34451394805</v>
       </c>
       <c r="H6" t="n">
         <v>0.4668095707893372</v>
       </c>
       <c r="I6" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -631,22 +631,22 @@
         <v>29400</v>
       </c>
       <c r="D7" t="n">
-        <v>20017.98828125</v>
+        <v>12122.189453125</v>
       </c>
       <c r="E7" t="n">
-        <v>5.560552300347222</v>
+        <v>3.367274848090278</v>
       </c>
       <c r="F7" t="n">
-        <v>20311.01171875</v>
+        <v>14776.966796875</v>
       </c>
       <c r="G7" t="n">
-        <v>17836.46986039677</v>
+        <v>9509.956615767867</v>
       </c>
       <c r="H7" t="n">
         <v>0.3423601686954498</v>
       </c>
       <c r="I7" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
03 v15: Mixup + BiLSTM score loss 일찍 (ep 10) → 0.6478 (+49%)
핵심 변경 (v11 → v15):
- Mixup augmentation (prob 0.3, beta α=0.2): 인접 측정 가중평균으로 데이터 증강
- BiLSTM score loss start ep 10 (TFT는 ep 30 유지): BiLSTM 학습 빠른 특성 보완
- AugDS 클래스에 Mixup 통합

베어링별 (v11 → v15):
- Train1: 0.7415 → 0.7584 (+2.3%) ★
- Train2: 0.7257 → 0.7295 (+0.5%) ★
- Train3: 0.5712 → 0.5590 (-2.1%)
- Train4: 0.5304 → 0.5444 (+2.6%) ★

평균: 0.6422 → 0.6478 (+0.9%)
RMSE: 10521 → 10155s (-3.5%)

Test1-6 submission.xlsx 재생성 (40 모델)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_김현우_Ensemble/results/submission.xlsx
+++ b/03_김현우_Ensemble/results/submission.xlsx
@@ -476,16 +476,16 @@
         <v>29400</v>
       </c>
       <c r="D2" t="n">
-        <v>32081.17578125</v>
+        <v>31309.81640625</v>
       </c>
       <c r="E2" t="n">
-        <v>8.911437717013889</v>
+        <v>8.697171223958334</v>
       </c>
       <c r="F2" t="n">
-        <v>34867.28125</v>
+        <v>34031.97265625</v>
       </c>
       <c r="G2" t="n">
-        <v>30276.91260032648</v>
+        <v>29525.92804222101</v>
       </c>
       <c r="H2" t="n">
         <v>0.221550315618515</v>
@@ -507,16 +507,16 @@
         <v>29400</v>
       </c>
       <c r="D3" t="n">
-        <v>33519.3515625</v>
+        <v>32040.50390625</v>
       </c>
       <c r="E3" t="n">
-        <v>9.310930989583333</v>
+        <v>8.900139973958334</v>
       </c>
       <c r="F3" t="n">
-        <v>35668.32421875</v>
+        <v>34442.2578125</v>
       </c>
       <c r="G3" t="n">
-        <v>31644.05439031613</v>
+        <v>30134.53174627316</v>
       </c>
       <c r="H3" t="n">
         <v>0.4320329427719116</v>
@@ -538,16 +538,16 @@
         <v>29400</v>
       </c>
       <c r="D4" t="n">
-        <v>7778.1416015625</v>
+        <v>6528.830078125</v>
       </c>
       <c r="E4" t="n">
-        <v>2.160594889322917</v>
+        <v>1.813563910590278</v>
       </c>
       <c r="F4" t="n">
-        <v>10197.79296875</v>
+        <v>9391.94140625</v>
       </c>
       <c r="G4" t="n">
-        <v>5724.486884062712</v>
+        <v>4536.519354765837</v>
       </c>
       <c r="H4" t="n">
         <v>0.2467963695526123</v>
@@ -569,16 +569,16 @@
         <v>29400</v>
       </c>
       <c r="D5" t="n">
-        <v>14910.0341796875</v>
+        <v>16029.5205078125</v>
       </c>
       <c r="E5" t="n">
-        <v>4.141676161024305</v>
+        <v>4.452644585503473</v>
       </c>
       <c r="F5" t="n">
-        <v>18841.48828125</v>
+        <v>18945.71484375</v>
       </c>
       <c r="G5" t="n">
-        <v>13105.61029044132</v>
+        <v>14259.53015128116</v>
       </c>
       <c r="H5" t="n">
         <v>0.03627244010567665</v>
@@ -600,16 +600,16 @@
         <v>29400</v>
       </c>
       <c r="D6" t="n">
-        <v>15525.8984375</v>
+        <v>15958.5546875</v>
       </c>
       <c r="E6" t="n">
-        <v>4.312749565972222</v>
+        <v>4.432931857638889</v>
       </c>
       <c r="F6" t="n">
-        <v>17378.8828125</v>
+        <v>17511.533203125</v>
       </c>
       <c r="G6" t="n">
-        <v>13562.34451394805</v>
+        <v>14153.42923074492</v>
       </c>
       <c r="H6" t="n">
         <v>0.4668095707893372</v>
@@ -631,16 +631,16 @@
         <v>29400</v>
       </c>
       <c r="D7" t="n">
-        <v>12122.189453125</v>
+        <v>11988.783203125</v>
       </c>
       <c r="E7" t="n">
-        <v>3.367274848090278</v>
+        <v>3.330217556423611</v>
       </c>
       <c r="F7" t="n">
-        <v>14776.966796875</v>
+        <v>17769.248046875</v>
       </c>
       <c r="G7" t="n">
-        <v>9509.956615767867</v>
+        <v>9109.094555220992</v>
       </c>
       <c r="H7" t="n">
         <v>0.3423601686954498</v>

</xml_diff>

<commit_message>
03 v17: late-RUL sample weight 2.0 → 0.6560 (+51%)
핵심 변경 (v15 → v17):
- AugDS에 sample weight 추가: 학습 데이터 마지막 30% RUL 측정에 weight 2.0
- 열화 진행 부분 (RUL 짧음 = FPT 이후) 학습 집중
- combined_loss에서 weighted MSE 적용

베어링별 (v15 → v17):
- Train1: 0.7584 → 0.7649 (+0.9%) median
- Train2: 0.7295 → 0.7557 (+3.6%) median ★
- Train3: 0.5590 → 0.5900 (+5.5%) ultra ★
- Train4: 0.5444 → 0.5438 (≈)

특히 Train3 (가장 어려운 베어링)에서 +5.5% 큰 개선:
- TFT 평균 0.388 → 0.439 (+13%)
- BiLSTM 평균 0.573 → 0.605 (+5.6%)

trim mean: 0.6478 → 0.6560 (+1.3%)
RMSE: 10155 → 9846s (-3%)

누적 (Train1+2+3) 평균: 0.7035 → 0.7 라인 돌파 (Train4가 평균 끌어내림)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_김현우_Ensemble/results/submission.xlsx
+++ b/03_김현우_Ensemble/results/submission.xlsx
@@ -476,16 +476,16 @@
         <v>29400</v>
       </c>
       <c r="D2" t="n">
-        <v>31309.81640625</v>
+        <v>32171.724609375</v>
       </c>
       <c r="E2" t="n">
-        <v>8.697171223958334</v>
+        <v>8.936590169270833</v>
       </c>
       <c r="F2" t="n">
-        <v>34031.97265625</v>
+        <v>34036.46484375</v>
       </c>
       <c r="G2" t="n">
-        <v>29525.92804222101</v>
+        <v>30295.80761985773</v>
       </c>
       <c r="H2" t="n">
         <v>0.221550315618515</v>
@@ -507,16 +507,16 @@
         <v>29400</v>
       </c>
       <c r="D3" t="n">
-        <v>32040.50390625</v>
+        <v>33102.015625</v>
       </c>
       <c r="E3" t="n">
-        <v>8.900139973958334</v>
+        <v>9.195004340277778</v>
       </c>
       <c r="F3" t="n">
-        <v>34442.2578125</v>
+        <v>34696.6171875</v>
       </c>
       <c r="G3" t="n">
-        <v>30134.53174627316</v>
+        <v>31155.85688055051</v>
       </c>
       <c r="H3" t="n">
         <v>0.4320329427719116</v>
@@ -538,16 +538,16 @@
         <v>29400</v>
       </c>
       <c r="D4" t="n">
-        <v>6528.830078125</v>
+        <v>7008.36669921875</v>
       </c>
       <c r="E4" t="n">
-        <v>1.813563910590278</v>
+        <v>1.946768527560764</v>
       </c>
       <c r="F4" t="n">
-        <v>9391.94140625</v>
+        <v>8994.220703125</v>
       </c>
       <c r="G4" t="n">
-        <v>4536.519354765837</v>
+        <v>5128.783026640837</v>
       </c>
       <c r="H4" t="n">
         <v>0.2467963695526123</v>
@@ -569,16 +569,16 @@
         <v>29400</v>
       </c>
       <c r="D5" t="n">
-        <v>16029.5205078125</v>
+        <v>15206.080078125</v>
       </c>
       <c r="E5" t="n">
-        <v>4.452644585503473</v>
+        <v>4.2239111328125</v>
       </c>
       <c r="F5" t="n">
-        <v>18945.71484375</v>
+        <v>17584.29296875</v>
       </c>
       <c r="G5" t="n">
-        <v>14259.53015128116</v>
+        <v>13426.87927237491</v>
       </c>
       <c r="H5" t="n">
         <v>0.03627244010567665</v>
@@ -600,16 +600,16 @@
         <v>29400</v>
       </c>
       <c r="D6" t="n">
-        <v>15958.5546875</v>
+        <v>14928.185546875</v>
       </c>
       <c r="E6" t="n">
-        <v>4.432931857638889</v>
+        <v>4.146718207465278</v>
       </c>
       <c r="F6" t="n">
-        <v>17511.533203125</v>
+        <v>15904.287109375</v>
       </c>
       <c r="G6" t="n">
-        <v>14153.42923074492</v>
+        <v>13068.38809304961</v>
       </c>
       <c r="H6" t="n">
         <v>0.4668095707893372</v>
@@ -631,16 +631,16 @@
         <v>29400</v>
       </c>
       <c r="D7" t="n">
-        <v>11988.783203125</v>
+        <v>11515.767578125</v>
       </c>
       <c r="E7" t="n">
-        <v>3.330217556423611</v>
+        <v>3.198824327256944</v>
       </c>
       <c r="F7" t="n">
-        <v>17769.248046875</v>
+        <v>16398.78515625</v>
       </c>
       <c r="G7" t="n">
-        <v>9109.094555220992</v>
+        <v>8683.539135299117</v>
       </c>
       <c r="H7" t="n">
         <v>0.3423601686954498</v>

</xml_diff>